<commit_message>
Radar: datos de 2026-09-12
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -205,14 +205,14 @@
     <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1066,10 +1066,10 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="13" t="n">
         <v>46277</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="12" t="n">
         <v>81.36</v>
       </c>
       <c r="J17" s="14">
@@ -1088,22 +1088,19 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E18" s="19">
-        <f>AVERAGE(E6:E17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="20" t="inlineStr">
+      <c r="D18" s="16" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>82.93000000000001</v>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="K18" s="21">
-        <f>E18</f>
+      <c r="K18" s="19">
+        <f>E19</f>
         <v/>
       </c>
     </row>
@@ -1114,10 +1111,14 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E19" s="21">
+        <f>AVERAGE(E6:E18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1127,6 +1128,11 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1459,9 +1465,9 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D19:H19"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1473,7 +1479,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E17">
+  <conditionalFormatting sqref="E6:E18">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1757,7 +1763,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E18</f>
+        <f>MIBGAS_Spot!E19</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-13
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -199,16 +199,16 @@
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1088,19 +1088,19 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="16" t="n">
+      <c r="D18" s="13" t="n">
         <v>46278</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="12" t="n">
         <v>82.93000000000001</v>
       </c>
-      <c r="J18" s="18" t="inlineStr">
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="K18" s="19">
-        <f>E19</f>
+      <c r="K18" s="17">
+        <f>E20</f>
         <v/>
       </c>
     </row>
@@ -1111,14 +1111,11 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E19" s="21">
-        <f>AVERAGE(E6:E18)</f>
-        <v/>
+      <c r="D19" s="18" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>84.95999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -1128,10 +1125,14 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E20" s="21">
+        <f>AVERAGE(E6:E19)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1141,6 +1142,11 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1464,8 +1470,8 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D21:H21"/>
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D20:H20"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
@@ -1479,7 +1485,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E18">
+  <conditionalFormatting sqref="E6:E19">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1763,7 +1769,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E19</f>
+        <f>MIBGAS_Spot!E20</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-14
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E20</f>
+        <f>E21</f>
         <v/>
       </c>
     </row>
@@ -1111,10 +1111,10 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="13" t="n">
         <v>46279</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="12" t="n">
         <v>84.95999999999999</v>
       </c>
     </row>
@@ -1125,14 +1125,11 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E20" s="21">
-        <f>AVERAGE(E6:E19)</f>
-        <v/>
+      <c r="D20" s="18" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1142,10 +1139,14 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E21" s="21">
+        <f>AVERAGE(E6:E20)</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1155,6 +1156,11 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1470,12 +1476,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D21:H21"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1485,7 +1491,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E19">
+  <conditionalFormatting sqref="E6:E20">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1543,7 +1549,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1575,7 +1581,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>79.97</v>
+        <v>83.38</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1593,7 +1599,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>79.64</v>
+        <v>83.05</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1611,7 +1617,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>79.65000000000001</v>
+        <v>82.66</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1629,7 +1635,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>79.93000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1647,7 +1653,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>77.58</v>
+        <v>82.53</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1665,7 +1671,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>56.07</v>
+        <v>56.76</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1678,7 +1684,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.44</v>
+        <v>51.41</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1691,7 +1697,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>53.74</v>
+        <v>54.07</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1704,7 +1710,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>78.43000000000001</v>
+        <v>82.33</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1717,7 +1723,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>58.83</v>
+        <v>60.18</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1730,7 +1736,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.17</v>
+        <v>35.87</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1769,7 +1775,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E20</f>
+        <f>MIBGAS_Spot!E21</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-15
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E21</f>
+        <f>E22</f>
         <v/>
       </c>
     </row>
@@ -1125,10 +1125,10 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="13" t="n">
         <v>46280</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="12" t="n">
         <v>85.70999999999999</v>
       </c>
     </row>
@@ -1139,14 +1139,11 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E21" s="21">
-        <f>AVERAGE(E6:E20)</f>
-        <v/>
+      <c r="D21" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>83.09999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -1156,10 +1153,14 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E22" s="21">
+        <f>AVERAGE(E6:E21)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1168,6 +1169,11 @@
       </c>
       <c r="B23" s="12" t="n">
         <v>34.55</v>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1480,8 +1486,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D23:H23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1491,7 +1497,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E20">
+  <conditionalFormatting sqref="E6:E21">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1549,7 +1555,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1581,7 +1587,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>83.38</v>
+        <v>81.38</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1599,7 +1605,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>83.05</v>
+        <v>80.28</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1617,7 +1623,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>82.66</v>
+        <v>80.06</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1635,7 +1641,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>83.59999999999999</v>
+        <v>81.55</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1653,7 +1659,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>82.53</v>
+        <v>77.36</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1671,7 +1677,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>56.76</v>
+        <v>55.09</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1684,7 +1690,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.41</v>
+        <v>50.06</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1697,7 +1703,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>54.07</v>
+        <v>52.56</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1710,7 +1716,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>82.33</v>
+        <v>77.93000000000001</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1723,7 +1729,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>60.18</v>
+        <v>57.83</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1736,7 +1742,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>35.87</v>
+        <v>35.5</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1775,7 +1781,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E21</f>
+        <f>MIBGAS_Spot!E22</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-16
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E22</f>
+        <f>E23</f>
         <v/>
       </c>
     </row>
@@ -1139,10 +1139,10 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="13" t="n">
         <v>46281</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="12" t="n">
         <v>83.09999999999999</v>
       </c>
     </row>
@@ -1153,14 +1153,11 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E22" s="21">
-        <f>AVERAGE(E6:E21)</f>
-        <v/>
+      <c r="D22" s="18" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>80.23999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1170,10 +1167,14 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E23" s="21">
+        <f>AVERAGE(E6:E22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1182,6 +1183,11 @@
       </c>
       <c r="B24" s="12" t="n">
         <v>32.42</v>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1484,9 +1490,9 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D23:H23"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1497,7 +1503,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E21">
+  <conditionalFormatting sqref="E6:E22">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1555,7 +1561,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1587,7 +1593,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>81.38</v>
+        <v>80.04000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1605,7 +1611,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>80.28</v>
+        <v>78</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1623,7 +1629,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>80.06</v>
+        <v>79</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1641,7 +1647,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>81.55</v>
+        <v>80</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>77.36</v>
+        <v>75.63</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>55.09</v>
+        <v>56.48</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1690,7 +1696,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>50.06</v>
+        <v>51.84</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>52.56</v>
+        <v>54.15</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1716,7 +1722,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>77.93000000000001</v>
+        <v>76.47</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1729,7 +1735,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>57.83</v>
+        <v>58.63</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1742,7 +1748,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>35.5</v>
+        <v>36.77</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1781,7 +1787,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E22</f>
+        <f>MIBGAS_Spot!E23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-17
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E23</f>
+        <f>E24</f>
         <v/>
       </c>
     </row>
@@ -1153,10 +1153,10 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="13" t="n">
         <v>46282</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="12" t="n">
         <v>80.23999999999999</v>
       </c>
     </row>
@@ -1167,14 +1167,11 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E23" s="21">
-        <f>AVERAGE(E6:E22)</f>
-        <v/>
+      <c r="D23" s="18" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>78.81</v>
       </c>
     </row>
     <row r="24">
@@ -1184,10 +1181,14 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E24" s="21">
+        <f>AVERAGE(E6:E23)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1197,6 +1198,11 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1489,8 +1495,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D25:H25"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1503,7 +1509,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E22">
+  <conditionalFormatting sqref="E6:E23">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1561,7 +1567,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1593,7 +1599,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>80.04000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1611,7 +1617,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>78</v>
+        <v>75.48999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1629,7 +1635,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>79</v>
+        <v>75.5</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1647,7 +1653,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>80</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1665,7 +1671,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>75.63</v>
+        <v>76.13</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1683,7 +1689,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>56.48</v>
+        <v>53.41</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1696,7 +1702,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.84</v>
+        <v>49.18</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1709,7 +1715,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>54.15</v>
+        <v>51.28</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1722,7 +1728,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>76.47</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1735,7 +1741,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>58.63</v>
+        <v>56.73</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1748,7 +1754,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.77</v>
+        <v>36.85</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1787,7 +1793,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E23</f>
+        <f>MIBGAS_Spot!E24</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-18
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E24</f>
+        <f>E25</f>
         <v/>
       </c>
     </row>
@@ -1167,10 +1167,10 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="18" t="n">
+      <c r="D23" s="13" t="n">
         <v>46283</v>
       </c>
-      <c r="E23" s="19" t="n">
+      <c r="E23" s="12" t="n">
         <v>78.81</v>
       </c>
     </row>
@@ -1181,14 +1181,11 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E24" s="21">
-        <f>AVERAGE(E6:E23)</f>
-        <v/>
+      <c r="D24" s="18" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>81.95999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1198,10 +1195,14 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E25" s="21">
+        <f>AVERAGE(E6:E24)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1211,6 +1212,11 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1495,11 +1501,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D25:H25"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1509,7 +1515,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E23">
+  <conditionalFormatting sqref="E6:E24">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1567,7 +1573,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1599,7 +1605,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>78.23999999999999</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1617,7 +1623,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>75.48999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1635,7 +1641,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>75.5</v>
+        <v>76.11</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1653,7 +1659,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>78.15000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1671,7 +1677,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>76.13</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1689,7 +1695,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>53.41</v>
+        <v>55.84</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1702,7 +1708,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>49.18</v>
+        <v>51.43</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1715,7 +1721,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>51.28</v>
+        <v>53.62</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1728,7 +1734,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>75.93000000000001</v>
+        <v>76.88</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1741,7 +1747,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>56.73</v>
+        <v>59</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1754,7 +1760,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.85</v>
+        <v>37</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1793,7 +1799,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E24</f>
+        <f>MIBGAS_Spot!E25</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-19
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E25</f>
+        <f>E26</f>
         <v/>
       </c>
     </row>
@@ -1181,10 +1181,10 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="13" t="n">
         <v>46284</v>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E24" s="12" t="n">
         <v>81.95999999999999</v>
       </c>
     </row>
@@ -1195,14 +1195,11 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E25" s="21">
-        <f>AVERAGE(E6:E24)</f>
-        <v/>
+      <c r="D25" s="18" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>81.2</v>
       </c>
     </row>
     <row r="26">
@@ -1212,10 +1209,14 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E26" s="21">
+        <f>AVERAGE(E6:E25)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1224,6 +1225,11 @@
       </c>
       <c r="B27" s="12" t="n">
         <v>40.41</v>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1504,8 +1510,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D27:H27"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1515,7 +1521,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E24">
+  <conditionalFormatting sqref="E6:E25">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1799,7 +1805,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E25</f>
+        <f>MIBGAS_Spot!E26</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-20
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E26</f>
+        <f>E27</f>
         <v/>
       </c>
     </row>
@@ -1195,10 +1195,10 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="13" t="n">
         <v>46285</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="12" t="n">
         <v>81.2</v>
       </c>
     </row>
@@ -1209,14 +1209,11 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E26" s="21">
-        <f>AVERAGE(E6:E25)</f>
-        <v/>
+      <c r="D26" s="18" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>83.8</v>
       </c>
     </row>
     <row r="27">
@@ -1226,10 +1223,14 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E27" s="21">
+        <f>AVERAGE(E6:E26)</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1238,6 +1239,11 @@
       </c>
       <c r="B28" s="12" t="n">
         <v>44.16</v>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1509,8 +1515,8 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D28:H28"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D27:H27"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1521,7 +1527,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E25">
+  <conditionalFormatting sqref="E6:E26">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1805,7 +1811,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E26</f>
+        <f>MIBGAS_Spot!E27</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-21
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E27</f>
+        <f>E28</f>
         <v/>
       </c>
     </row>
@@ -1209,10 +1209,10 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="18" t="n">
+      <c r="D26" s="13" t="n">
         <v>46286</v>
       </c>
-      <c r="E26" s="19" t="n">
+      <c r="E26" s="12" t="n">
         <v>83.8</v>
       </c>
     </row>
@@ -1223,14 +1223,11 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E27" s="21">
-        <f>AVERAGE(E6:E26)</f>
-        <v/>
+      <c r="D27" s="18" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>75.53</v>
       </c>
     </row>
     <row r="28">
@@ -1240,10 +1237,14 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E28" s="21">
+        <f>AVERAGE(E6:E27)</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1252,6 +1253,11 @@
       </c>
       <c r="B29" s="12" t="n">
         <v>46.23</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1515,8 +1521,8 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D28:H28"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1527,7 +1533,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E26">
+  <conditionalFormatting sqref="E6:E27">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1585,7 +1591,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1617,7 +1623,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>77.98999999999999</v>
+        <v>74.83</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1635,7 +1641,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>78.09999999999999</v>
+        <v>72.58</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1653,7 +1659,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>76.11</v>
+        <v>75.2</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1671,7 +1677,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>77.8</v>
+        <v>72.77</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1689,7 +1695,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>75.90000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1707,7 +1713,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>55.84</v>
+        <v>55.65</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1720,7 +1726,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.43</v>
+        <v>51.78</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1733,7 +1739,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>53.62</v>
+        <v>53.7</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1746,7 +1752,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>76.88</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1759,7 +1765,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>59</v>
+        <v>57.28</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1772,7 +1778,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>37</v>
+        <v>37.33</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1811,7 +1817,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E27</f>
+        <f>MIBGAS_Spot!E28</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-22
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E28</f>
+        <f>E29</f>
         <v/>
       </c>
     </row>
@@ -1223,10 +1223,10 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="13" t="n">
         <v>46287</v>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E27" s="12" t="n">
         <v>75.53</v>
       </c>
     </row>
@@ -1237,14 +1237,11 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E28" s="21">
-        <f>AVERAGE(E6:E27)</f>
-        <v/>
+      <c r="D28" s="18" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>75.41</v>
       </c>
     </row>
     <row r="29">
@@ -1254,10 +1251,14 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E29" s="21">
+        <f>AVERAGE(E6:E28)</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1267,6 +1268,11 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -1518,11 +1524,11 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D30:H30"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1533,7 +1539,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E27">
+  <conditionalFormatting sqref="E6:E28">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1591,7 +1597,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1623,7 +1629,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>74.83</v>
+        <v>71.51000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1641,7 +1647,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>72.58</v>
+        <v>71</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>75.2</v>
+        <v>69.44</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>72.77</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1695,7 +1701,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>70.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1713,7 +1719,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>55.65</v>
+        <v>54.31</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1726,7 +1732,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.78</v>
+        <v>50.67</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1739,7 +1745,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>53.7</v>
+        <v>52.48</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1752,7 +1758,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>71.84999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1765,7 +1771,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>57.28</v>
+        <v>56.6</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1778,7 +1784,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>37.33</v>
+        <v>36.54</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1817,7 +1823,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E28</f>
+        <f>MIBGAS_Spot!E29</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-23
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E29</f>
+        <f>E30</f>
         <v/>
       </c>
     </row>
@@ -1237,10 +1237,10 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="18" t="n">
+      <c r="D28" s="13" t="n">
         <v>46288</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="12" t="n">
         <v>75.41</v>
       </c>
     </row>
@@ -1251,14 +1251,11 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E29" s="21">
-        <f>AVERAGE(E6:E28)</f>
-        <v/>
+      <c r="D29" s="18" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E29" s="19" t="n">
+        <v>74.33</v>
       </c>
     </row>
     <row r="30">
@@ -1268,10 +1265,14 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E30" s="21">
+        <f>AVERAGE(E6:E29)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1281,6 +1282,11 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1524,12 +1530,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D30:H30"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1539,7 +1545,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E28">
+  <conditionalFormatting sqref="E6:E29">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1597,7 +1603,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1629,7 +1635,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>71.51000000000001</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1647,7 +1653,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>71</v>
+        <v>72.48</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1665,7 +1671,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>69.44</v>
+        <v>72.19</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1683,7 +1689,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>70.90000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1701,7 +1707,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>68.5</v>
+        <v>70.23</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1719,7 +1725,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>54.31</v>
+        <v>54.15</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1732,7 +1738,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>50.67</v>
+        <v>50.55</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1745,7 +1751,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>52.48</v>
+        <v>52.34</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1758,7 +1764,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>69.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1784,7 +1790,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.54</v>
+        <v>36.91</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1823,7 +1829,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E29</f>
+        <f>MIBGAS_Spot!E30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-24
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E30</f>
+        <f>E31</f>
         <v/>
       </c>
     </row>
@@ -1251,10 +1251,10 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="18" t="n">
+      <c r="D29" s="13" t="n">
         <v>46289</v>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E29" s="12" t="n">
         <v>74.33</v>
       </c>
     </row>
@@ -1265,14 +1265,11 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E30" s="21">
-        <f>AVERAGE(E6:E29)</f>
-        <v/>
+      <c r="D30" s="18" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E30" s="19" t="n">
+        <v>76.56</v>
       </c>
     </row>
     <row r="31">
@@ -1282,10 +1279,14 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E31" s="21">
+        <f>AVERAGE(E6:E30)</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1294,6 +1295,11 @@
       </c>
       <c r="B32" s="12" t="n">
         <v>41.41</v>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1535,7 +1541,7 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1545,7 +1551,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E29">
+  <conditionalFormatting sqref="E6:E30">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1603,7 +1609,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1635,7 +1641,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>72.34999999999999</v>
+        <v>74.13</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1653,7 +1659,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>72.48</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1671,7 +1677,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>72.19</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1689,7 +1695,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>71.7</v>
+        <v>74.2</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1707,7 +1713,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>70.23</v>
+        <v>73.41</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1725,7 +1731,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>54.15</v>
+        <v>55.85</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1738,7 +1744,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>50.55</v>
+        <v>51.89</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1751,7 +1757,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>52.34</v>
+        <v>53.86</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1764,7 +1770,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>71.09999999999999</v>
+        <v>74.13</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1777,7 +1783,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>56.6</v>
+        <v>58</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1790,7 +1796,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.91</v>
+        <v>37.7</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1829,7 +1835,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E30</f>
+        <f>MIBGAS_Spot!E31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-25
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E31</f>
+        <f>E32</f>
         <v/>
       </c>
     </row>
@@ -1265,10 +1265,10 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="13" t="n">
         <v>46290</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="12" t="n">
         <v>76.56</v>
       </c>
     </row>
@@ -1279,14 +1279,11 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E31" s="21">
-        <f>AVERAGE(E6:E30)</f>
-        <v/>
+      <c r="D31" s="18" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>73.12</v>
       </c>
     </row>
     <row r="32">
@@ -1296,10 +1293,14 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E32" s="21">
+        <f>AVERAGE(E6:E31)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1308,6 +1309,11 @@
       </c>
       <c r="B33" s="12" t="n">
         <v>33.76</v>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1539,9 +1545,9 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D33:H33"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D32:H32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1551,7 +1557,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E30">
+  <conditionalFormatting sqref="E6:E31">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1609,7 +1615,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1641,7 +1647,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>74.13</v>
+        <v>71.94</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>73.76000000000001</v>
+        <v>70.84999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>73.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1695,7 +1701,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>74.2</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1713,7 +1719,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>73.41</v>
+        <v>69.06</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1731,7 +1737,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>55.85</v>
+        <v>54</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1744,7 +1750,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.89</v>
+        <v>50.49</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1757,7 +1763,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>53.86</v>
+        <v>52.23</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1770,7 +1776,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>74.13</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1783,7 +1789,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>58</v>
+        <v>55.75</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1796,7 +1802,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>37.7</v>
+        <v>36.94</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1835,7 +1841,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E31</f>
+        <f>MIBGAS_Spot!E32</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-26
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E32</f>
+        <f>E33</f>
         <v/>
       </c>
     </row>
@@ -1279,10 +1279,10 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="13" t="n">
         <v>46291</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="12" t="n">
         <v>73.12</v>
       </c>
     </row>
@@ -1293,14 +1293,11 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E32" s="21">
-        <f>AVERAGE(E6:E31)</f>
-        <v/>
+      <c r="D32" s="18" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>72.66</v>
       </c>
     </row>
     <row r="33">
@@ -1310,10 +1307,14 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E33" s="21">
+        <f>AVERAGE(E6:E32)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1322,6 +1323,11 @@
       </c>
       <c r="B34" s="12" t="n">
         <v>34.02</v>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1544,8 +1550,8 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D34:H34"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D33:H33"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1557,7 +1563,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E31">
+  <conditionalFormatting sqref="E6:E32">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1841,7 +1847,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E32</f>
+        <f>MIBGAS_Spot!E33</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-27
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E33</f>
+        <f>E34</f>
         <v/>
       </c>
     </row>
@@ -1293,10 +1293,10 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="18" t="n">
+      <c r="D32" s="13" t="n">
         <v>46292</v>
       </c>
-      <c r="E32" s="19" t="n">
+      <c r="E32" s="12" t="n">
         <v>72.66</v>
       </c>
     </row>
@@ -1307,14 +1307,11 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E33" s="21">
-        <f>AVERAGE(E6:E32)</f>
-        <v/>
+      <c r="D33" s="18" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E33" s="19" t="n">
+        <v>75.25</v>
       </c>
     </row>
     <row r="34">
@@ -1324,10 +1321,14 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D34" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E34" s="21">
+        <f>AVERAGE(E6:E33)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -1337,6 +1338,11 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1548,9 +1554,9 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D35:H35"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D34:H34"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1563,7 +1569,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E32">
+  <conditionalFormatting sqref="E6:E33">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1847,7 +1853,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E33</f>
+        <f>MIBGAS_Spot!E34</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-28
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E34</f>
+        <f>E35</f>
         <v/>
       </c>
     </row>
@@ -1307,10 +1307,10 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="18" t="n">
+      <c r="D33" s="13" t="n">
         <v>46293</v>
       </c>
-      <c r="E33" s="19" t="n">
+      <c r="E33" s="12" t="n">
         <v>75.25</v>
       </c>
     </row>
@@ -1321,14 +1321,11 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E34" s="21">
-        <f>AVERAGE(E6:E33)</f>
-        <v/>
+      <c r="D34" s="18" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <v>74.87</v>
       </c>
     </row>
     <row r="35">
@@ -1338,10 +1335,14 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D35" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E35" s="21">
+        <f>AVERAGE(E6:E34)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -1351,6 +1352,11 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1554,12 +1560,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D35:H35"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D36:H36"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1569,7 +1575,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E33">
+  <conditionalFormatting sqref="E6:E34">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1627,7 +1633,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>71.94</v>
+        <v>73.03</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>70.84999999999999</v>
+        <v>73.33</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1713,7 +1719,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>70.40000000000001</v>
+        <v>73.25</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1731,7 +1737,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>69.06</v>
+        <v>71.56</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1749,7 +1755,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>54</v>
+        <v>54.7</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1762,7 +1768,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>50.49</v>
+        <v>50.91</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1775,7 +1781,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>52.23</v>
+        <v>52.8</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1788,7 +1794,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>70.15000000000001</v>
+        <v>72.13</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1801,7 +1807,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>55.75</v>
+        <v>56.73</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1814,7 +1820,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.94</v>
+        <v>37.02</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1853,7 +1859,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E34</f>
+        <f>MIBGAS_Spot!E35</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-29
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -203,12 +203,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1321,10 +1315,10 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="18" t="n">
+      <c r="D34" s="13" t="n">
         <v>46294</v>
       </c>
-      <c r="E34" s="19" t="n">
+      <c r="E34" s="12" t="n">
         <v>74.87</v>
       </c>
     </row>
@@ -1335,12 +1329,12 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D35" s="18" t="inlineStr">
         <is>
           <t>MEDIA MES</t>
         </is>
       </c>
-      <c r="E35" s="21">
+      <c r="E35" s="19">
         <f>AVERAGE(E6:E34)</f>
         <v/>
       </c>
@@ -1352,7 +1346,7 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="22" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
         </is>
@@ -1466,97 +1460,97 @@
       <c r="A50" s="11" t="n">
         <v>46266</v>
       </c>
-      <c r="B50" s="23" t="n"/>
+      <c r="B50" s="21" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="23" t="n"/>
+      <c r="B51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="23" t="n"/>
+      <c r="B52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="23" t="n"/>
+      <c r="B53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="23" t="n"/>
+      <c r="B56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="23" t="n"/>
+      <c r="B57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="23" t="n"/>
+      <c r="B58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="23" t="n"/>
+      <c r="B59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="23" t="n"/>
+      <c r="B60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="23" t="n"/>
+      <c r="B61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="23" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="23" t="n"/>
+      <c r="B63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="23" t="n"/>
+      <c r="B64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="23" t="n"/>
+      <c r="B65" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1627,12 +1621,12 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="23" t="n">
         <v>46293</v>
       </c>
     </row>
@@ -1659,217 +1653,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Mes M+1 (Oct26-Oct26)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="25" t="n">
         <v>73.03</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Mes M+2 (Nov26-Nov26)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="25" t="n">
         <v>73.33</v>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Mes M+3 (Dec26-Dec26)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="25" t="n">
         <v>72.2</v>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Oct26-Dec26)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="25" t="n">
         <v>73.25</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
+      <c r="B10" s="25" t="n">
         <v>71.56</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="25" t="n">
         <v>54.7</v>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="25" t="n">
         <v>50.91</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
+      <c r="B13" s="25" t="n">
         <v>52.8</v>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct26-Mar27)</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
+      <c r="B14" s="25" t="n">
         <v>72.13</v>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
+      <c r="B15" s="25" t="n">
         <v>56.73</v>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
+      <c r="B16" s="25" t="n">
         <v>37.02</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="22">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="33">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="31">
         <f>MIBGAS_Spot!E35</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="31">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-30
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E35</f>
+        <f>E36</f>
         <v/>
       </c>
     </row>
@@ -1329,14 +1329,11 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E35" s="19">
-        <f>AVERAGE(E6:E34)</f>
-        <v/>
+      <c r="D35" s="13" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <v>70.41</v>
       </c>
     </row>
     <row r="36">
@@ -1346,10 +1343,14 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E36" s="19">
+        <f>AVERAGE(E6:E35)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1358,6 +1359,11 @@
       </c>
       <c r="B37" s="12" t="n">
         <v>32.58</v>
+      </c>
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1558,8 +1564,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D37:H37"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D36:H36"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1569,7 +1575,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E34">
+  <conditionalFormatting sqref="E6:E35">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1627,7 +1633,7 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>73.03</v>
+        <v>70.97</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>0</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>73.33</v>
+        <v>71.89</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>0</v>
@@ -1695,7 +1701,7 @@
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>72.2</v>
+        <v>71</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>0</v>
@@ -1713,7 +1719,7 @@
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>73.25</v>
+        <v>69.3</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>3</v>
@@ -1731,7 +1737,7 @@
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>71.56</v>
+        <v>70.5</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>3</v>
@@ -1762,7 +1768,7 @@
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>50.91</v>
+        <v>50.88</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>3</v>
@@ -1775,7 +1781,7 @@
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>52.8</v>
+        <v>52.78</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>0</v>
@@ -1784,11 +1790,11 @@
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>Invierno (oct-mar) (Oct26-Mar27)</t>
+          <t>Invierno (oct-mar) (Oct27-Mar28)</t>
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>72.13</v>
+        <v>48.45</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>0</v>
@@ -1801,7 +1807,7 @@
         </is>
       </c>
       <c r="B15" s="25" t="n">
-        <v>56.73</v>
+        <v>56</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>0</v>
@@ -1814,7 +1820,7 @@
         </is>
       </c>
       <c r="B16" s="25" t="n">
-        <v>37.02</v>
+        <v>36.76</v>
       </c>
       <c r="C16" s="26" t="n">
         <v>0</v>
@@ -1853,7 +1859,7 @@
         </is>
       </c>
       <c r="B20" s="31">
-        <f>MIBGAS_Spot!E35</f>
+        <f>MIBGAS_Spot!E36</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-01
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -199,10 +199,10 @@
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,6 +210,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -770,7 +776,7 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>MES EN CURSO (Sep-2026)</t>
+          <t>MES EN CURSO (Oct-2026)</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
@@ -819,10 +825,10 @@
         <v>60.62</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>46266</v>
+        <v>46296</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>70.27</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="J6" s="14">
         <f>A42</f>
@@ -840,11 +846,11 @@
       <c r="B7" s="12" t="n">
         <v>52.17</v>
       </c>
-      <c r="D7" s="13" t="n">
-        <v>46267</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>72.48</v>
+      <c r="D7" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>73.77</v>
       </c>
       <c r="J7" s="14">
         <f>A43</f>
@@ -862,11 +868,14 @@
       <c r="B8" s="12" t="n">
         <v>43.67</v>
       </c>
-      <c r="D8" s="13" t="n">
-        <v>46268</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>73.91</v>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E8" s="19">
+        <f>AVERAGE(E6:E7)</f>
+        <v/>
       </c>
       <c r="J8" s="14">
         <f>A44</f>
@@ -884,11 +893,10 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="13" t="n">
-        <v>46269</v>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>72.09999999999999</v>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
       <c r="J9" s="14">
         <f>A45</f>
@@ -906,12 +914,6 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="13" t="n">
-        <v>46270</v>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>72.84999999999999</v>
-      </c>
       <c r="J10" s="14">
         <f>A46</f>
         <v/>
@@ -928,12 +930,6 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="13" t="n">
-        <v>46271</v>
-      </c>
-      <c r="E11" s="12" t="n">
-        <v>79.03</v>
-      </c>
       <c r="J11" s="14">
         <f>A47</f>
         <v/>
@@ -950,12 +946,6 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <v>46272</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>77.63</v>
-      </c>
       <c r="J12" s="14">
         <f>A48</f>
         <v/>
@@ -972,12 +962,6 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="13" t="n">
-        <v>46273</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>74.76000000000001</v>
-      </c>
       <c r="J13" s="14">
         <f>A49</f>
         <v/>
@@ -994,12 +978,6 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="13" t="n">
-        <v>46274</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>77.44</v>
-      </c>
       <c r="J14" s="14">
         <f>A50</f>
         <v/>
@@ -1016,12 +994,6 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="13" t="n">
-        <v>46275</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>80.77</v>
-      </c>
       <c r="J15" s="14">
         <f>A51</f>
         <v/>
@@ -1038,12 +1010,6 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="13" t="n">
-        <v>46276</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>83.45999999999999</v>
-      </c>
       <c r="J16" s="14">
         <f>A52</f>
         <v/>
@@ -1060,12 +1026,6 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="13" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>81.36</v>
-      </c>
       <c r="J17" s="14">
         <f>A53</f>
         <v/>
@@ -1082,19 +1042,13 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="13" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>82.93000000000001</v>
-      </c>
-      <c r="J18" s="16" t="inlineStr">
-        <is>
-          <t>Sep</t>
-        </is>
-      </c>
-      <c r="K18" s="17">
-        <f>E36</f>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="K18" s="22">
+        <f>E8</f>
         <v/>
       </c>
     </row>
@@ -1105,12 +1059,6 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="13" t="n">
-        <v>46279</v>
-      </c>
-      <c r="E19" s="12" t="n">
-        <v>84.95999999999999</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n">
@@ -1119,12 +1067,6 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="13" t="n">
-        <v>46280</v>
-      </c>
-      <c r="E20" s="12" t="n">
-        <v>85.70999999999999</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1133,12 +1075,6 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="13" t="n">
-        <v>46281</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>83.09999999999999</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1147,12 +1083,6 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="13" t="n">
-        <v>46282</v>
-      </c>
-      <c r="E22" s="12" t="n">
-        <v>80.23999999999999</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1161,12 +1091,6 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="13" t="n">
-        <v>46283</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>78.81</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
@@ -1175,12 +1099,6 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="13" t="n">
-        <v>46284</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <v>81.95999999999999</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
@@ -1189,12 +1107,6 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="13" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E25" s="12" t="n">
-        <v>81.2</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1203,12 +1115,6 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="13" t="n">
-        <v>46286</v>
-      </c>
-      <c r="E26" s="12" t="n">
-        <v>83.8</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1217,12 +1123,6 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="13" t="n">
-        <v>46287</v>
-      </c>
-      <c r="E27" s="12" t="n">
-        <v>75.53</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1231,12 +1131,6 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="13" t="n">
-        <v>46288</v>
-      </c>
-      <c r="E28" s="12" t="n">
-        <v>75.41</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n">
@@ -1245,12 +1139,6 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="13" t="n">
-        <v>46289</v>
-      </c>
-      <c r="E29" s="12" t="n">
-        <v>74.33</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1259,12 +1147,6 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="13" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E30" s="12" t="n">
-        <v>76.56</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -1273,12 +1155,6 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="13" t="n">
-        <v>46291</v>
-      </c>
-      <c r="E31" s="12" t="n">
-        <v>73.12</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1287,12 +1163,6 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="13" t="n">
-        <v>46292</v>
-      </c>
-      <c r="E32" s="12" t="n">
-        <v>72.66</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
@@ -1301,12 +1171,6 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="13" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E33" s="12" t="n">
-        <v>75.25</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -1315,12 +1179,6 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="13" t="n">
-        <v>46294</v>
-      </c>
-      <c r="E34" s="12" t="n">
-        <v>74.87</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n">
@@ -1329,12 +1187,6 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="13" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E35" s="12" t="n">
-        <v>70.41</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1343,15 +1195,6 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E36" s="19">
-        <f>AVERAGE(E6:E35)</f>
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1360,11 +1203,6 @@
       <c r="B37" s="12" t="n">
         <v>32.58</v>
       </c>
-      <c r="D37" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -1466,97 +1304,99 @@
       <c r="A50" s="11" t="n">
         <v>46266</v>
       </c>
-      <c r="B50" s="21" t="n"/>
+      <c r="B50" s="12" t="n">
+        <v>77.56</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="21" t="n"/>
+      <c r="B51" s="23" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="21" t="n"/>
+      <c r="B52" s="23" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="21" t="n"/>
+      <c r="B53" s="23" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="21" t="n"/>
+      <c r="B54" s="23" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="21" t="n"/>
+      <c r="B55" s="23" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="21" t="n"/>
+      <c r="B56" s="23" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="21" t="n"/>
+      <c r="B57" s="23" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="21" t="n"/>
+      <c r="B58" s="23" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="21" t="n"/>
+      <c r="B59" s="23" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="21" t="n"/>
+      <c r="B60" s="23" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="21" t="n"/>
+      <c r="B61" s="23" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="21" t="n"/>
+      <c r="B62" s="23" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="21" t="n"/>
+      <c r="B63" s="23" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="21" t="n"/>
+      <c r="B64" s="23" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="21" t="n"/>
+      <c r="B65" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1564,8 +1404,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D37:H37"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D9:H9"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1575,7 +1415,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E35">
+  <conditionalFormatting sqref="E6:E7">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1627,13 +1467,13 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
-        <v>46295</v>
+      <c r="B4" s="25" t="n">
+        <v>46296</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1659,217 +1499,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Mes M+1 (Oct26-Oct26)</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="n">
-        <v>70.97</v>
-      </c>
-      <c r="C6" s="26" t="n">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Mes M+1 (Nov26-Nov26)</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>73.08</v>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Mes M+2 (Dec26-Dec26)</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>73.05</v>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Mes M+3 (Jan27-Jan27)</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>72.98</v>
+      </c>
+      <c r="C8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="27" t="inlineStr">
-        <is>
-          <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>Mes M+2 (Nov26-Nov26)</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="n">
-        <v>71.89</v>
-      </c>
-      <c r="C7" s="26" t="n">
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Trimestre Q+1 (Jan27-Mar27)</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>71.23</v>
+      </c>
+      <c r="C9" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Trimestre Q+2 (Apr27-Jun27)</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>55.62</v>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Trimestre Q+3 (Jul27-Sep27)</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>51.66</v>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Trimestre Q+4 (Oct27-Dec27)</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="C12" s="28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Verano (abr-sep) (Apr27-Sep27)</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>54.05</v>
+      </c>
+      <c r="C13" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="27" t="inlineStr">
-        <is>
-          <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Mes M+3 (Dec26-Dec26)</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="n">
-        <v>71</v>
-      </c>
-      <c r="C8" s="26" t="n">
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>Invierno (oct-mar) (Oct27-Mar28)</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="C14" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="27" t="inlineStr">
-        <is>
-          <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>Trimestre Q+1 (Oct26-Dec26)</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n">
-        <v>69.3</v>
-      </c>
-      <c r="C9" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" s="27" t="inlineStr">
-        <is>
-          <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
-        <is>
-          <t>Trimestre Q+2 (Jan27-Mar27)</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>70.5</v>
-      </c>
-      <c r="C10" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" s="27" t="inlineStr">
-        <is>
-          <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t>Trimestre Q+3 (Apr27-Jun27)</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="C11" s="26" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t>Trimestre Q+4 (Jul27-Sep27)</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>50.88</v>
-      </c>
-      <c r="C12" s="26" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Verano (abr-sep) (Apr27-Sep27)</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>52.78</v>
-      </c>
-      <c r="C13" s="26" t="n">
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Año Y+1 (Jan27-Dec27)</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>57.35</v>
+      </c>
+      <c r="C15" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Invierno (oct-mar) (Oct27-Mar28)</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="n">
-        <v>48.45</v>
-      </c>
-      <c r="C14" s="26" t="n">
+    <row r="16">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Año Y+2 (Jan28-Dec28)</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="C16" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="29" t="inlineStr">
-        <is>
-          <t>Año Y+1 (Jan27-Dec27)</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="n">
-        <v>56</v>
-      </c>
-      <c r="C15" s="26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="29" t="inlineStr">
-        <is>
-          <t>Año Y+2 (Jan28-Dec28)</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="n">
-        <v>36.76</v>
-      </c>
-      <c r="C16" s="26" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="31">
+      <c r="B18" s="33">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="24">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="35">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="31">
-        <f>MIBGAS_Spot!E36</f>
+      <c r="B20" s="33">
+        <f>MIBGAS_Spot!E8</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="31">
+      <c r="B21" s="33">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-02
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -846,10 +846,10 @@
       <c r="B7" s="12" t="n">
         <v>52.17</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="13" t="n">
         <v>46297</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="12" t="n">
         <v>73.77</v>
       </c>
       <c r="J7" s="14">
@@ -868,14 +868,11 @@
       <c r="B8" s="12" t="n">
         <v>43.67</v>
       </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E8" s="19">
-        <f>AVERAGE(E6:E7)</f>
-        <v/>
+      <c r="D8" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>74.87</v>
       </c>
       <c r="J8" s="14">
         <f>A44</f>
@@ -893,10 +890,14 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E9" s="19">
+        <f>AVERAGE(E6:E8)</f>
+        <v/>
       </c>
       <c r="J9" s="14">
         <f>A45</f>
@@ -914,6 +915,11 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J10" s="14">
         <f>A46</f>
         <v/>
@@ -1048,7 +1054,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E8</f>
+        <f>E9</f>
         <v/>
       </c>
     </row>
@@ -1402,10 +1408,10 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D10:H10"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D9:H9"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1415,7 +1421,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E7">
+  <conditionalFormatting sqref="E6:E8">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1473,7 +1479,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1505,7 +1511,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>73.08</v>
+        <v>71.83</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1523,7 +1529,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>73.05</v>
+        <v>73.09</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1541,7 +1547,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>72.98</v>
+        <v>74.05</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1559,7 +1565,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>71.23</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1577,7 +1583,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>55.62</v>
+        <v>57.63</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1595,7 +1601,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>51.66</v>
+        <v>53.64</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1608,7 +1614,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>51.19</v>
+        <v>52.79</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1621,7 +1627,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>54.05</v>
+        <v>55.63</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1634,7 +1640,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>49.87</v>
+        <v>51.48</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1647,7 +1653,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>57.35</v>
+        <v>58.15</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1660,7 +1666,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>38.3</v>
+        <v>39.16</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1699,7 +1705,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E8</f>
+        <f>MIBGAS_Spot!E9</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-03
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -868,10 +868,10 @@
       <c r="B8" s="12" t="n">
         <v>43.67</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="13" t="n">
         <v>46298</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="12" t="n">
         <v>74.87</v>
       </c>
       <c r="J8" s="14">
@@ -890,14 +890,11 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E9" s="19">
-        <f>AVERAGE(E6:E8)</f>
-        <v/>
+      <c r="D9" s="16" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>78.09</v>
       </c>
       <c r="J9" s="14">
         <f>A45</f>
@@ -915,10 +912,14 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E10" s="19">
+        <f>AVERAGE(E6:E9)</f>
+        <v/>
       </c>
       <c r="J10" s="14">
         <f>A46</f>
@@ -936,6 +937,11 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J11" s="14">
         <f>A47</f>
         <v/>
@@ -1054,7 +1060,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E9</f>
+        <f>E10</f>
         <v/>
       </c>
     </row>
@@ -1408,8 +1414,8 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D10:H10"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D11:H11"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1421,7 +1427,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E8">
+  <conditionalFormatting sqref="E6:E9">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1705,7 +1711,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E9</f>
+        <f>MIBGAS_Spot!E10</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-04
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -890,10 +890,10 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="13" t="n">
         <v>46299</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="12" t="n">
         <v>78.09</v>
       </c>
       <c r="J9" s="14">
@@ -912,14 +912,11 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E10" s="19">
-        <f>AVERAGE(E6:E9)</f>
-        <v/>
+      <c r="D10" s="16" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>77.40000000000001</v>
       </c>
       <c r="J10" s="14">
         <f>A46</f>
@@ -937,10 +934,14 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E11" s="19">
+        <f>AVERAGE(E6:E10)</f>
+        <v/>
       </c>
       <c r="J11" s="14">
         <f>A47</f>
@@ -958,6 +959,11 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J12" s="14">
         <f>A48</f>
         <v/>
@@ -1060,7 +1066,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E10</f>
+        <f>E11</f>
         <v/>
       </c>
     </row>
@@ -1412,10 +1418,10 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D12:H12"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D11:H11"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1427,7 +1433,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E9">
+  <conditionalFormatting sqref="E6:E10">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1711,7 +1717,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E10</f>
+        <f>MIBGAS_Spot!E11</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-06
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -197,12 +197,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -912,10 +906,10 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="13" t="n">
         <v>46300</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="12" t="n">
         <v>77.40000000000001</v>
       </c>
       <c r="J10" s="14">
@@ -934,14 +928,11 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E11" s="19">
-        <f>AVERAGE(E6:E10)</f>
-        <v/>
+      <c r="D11" s="13" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>73.38</v>
       </c>
       <c r="J11" s="14">
         <f>A47</f>
@@ -959,10 +950,14 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E12" s="17">
+        <f>AVERAGE(E6:E11)</f>
+        <v/>
       </c>
       <c r="J12" s="14">
         <f>A48</f>
@@ -980,6 +975,11 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J13" s="14">
         <f>A49</f>
         <v/>
@@ -1060,13 +1060,13 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="J18" s="19" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="K18" s="22">
-        <f>E11</f>
+      <c r="K18" s="20">
+        <f>E12</f>
         <v/>
       </c>
     </row>
@@ -1330,98 +1330,98 @@
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="23" t="n"/>
+      <c r="B51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="23" t="n"/>
+      <c r="B52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="23" t="n"/>
+      <c r="B53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="23" t="n"/>
+      <c r="B56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="23" t="n"/>
+      <c r="B57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="23" t="n"/>
+      <c r="B58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="23" t="n"/>
+      <c r="B59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="23" t="n"/>
+      <c r="B60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="23" t="n"/>
+      <c r="B61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="23" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="23" t="n"/>
+      <c r="B63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="23" t="n"/>
+      <c r="B64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="23" t="n"/>
+      <c r="B65" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D12:H12"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D13:H13"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1433,7 +1433,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E10">
+  <conditionalFormatting sqref="E6:E11">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1485,13 +1485,13 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
-        <v>46297</v>
+      <c r="B4" s="23" t="n">
+        <v>46300</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1517,217 +1517,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Mes M+1 (Nov26-Nov26)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
-        <v>71.83</v>
-      </c>
-      <c r="C6" s="28" t="n">
+      <c r="B6" s="25" t="n">
+        <v>73.51000000000001</v>
+      </c>
+      <c r="C6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Mes M+2 (Dec26-Dec26)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
-        <v>73.09</v>
-      </c>
-      <c r="C7" s="28" t="n">
+      <c r="B7" s="25" t="n">
+        <v>72.92</v>
+      </c>
+      <c r="C7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Mes M+3 (Jan27-Jan27)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
-        <v>74.05</v>
-      </c>
-      <c r="C8" s="28" t="n">
+      <c r="B8" s="25" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="C8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
-        <v>72.15000000000001</v>
-      </c>
-      <c r="C9" s="28" t="n">
+      <c r="B9" s="25" t="n">
+        <v>72.05</v>
+      </c>
+      <c r="C9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
-        <v>57.63</v>
-      </c>
-      <c r="C10" s="28" t="n">
+      <c r="B10" s="25" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="C10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
-        <v>53.64</v>
-      </c>
-      <c r="C11" s="28" t="n">
+      <c r="B11" s="25" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="C11" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Oct27-Dec27)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
-        <v>52.79</v>
-      </c>
-      <c r="C12" s="28" t="n">
+      <c r="B12" s="25" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="C12" s="26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
-        <v>55.63</v>
-      </c>
-      <c r="C13" s="28" t="n">
+      <c r="B13" s="25" t="n">
+        <v>55.43</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct27-Mar28)</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
-        <v>51.48</v>
-      </c>
-      <c r="C14" s="28" t="n">
+      <c r="B14" s="25" t="n">
+        <v>51.32</v>
+      </c>
+      <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
-        <v>58.15</v>
-      </c>
-      <c r="C15" s="28" t="n">
+      <c r="B15" s="25" t="n">
+        <v>58.85</v>
+      </c>
+      <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
-        <v>39.16</v>
-      </c>
-      <c r="C16" s="28" t="n">
+      <c r="B16" s="25" t="n">
+        <v>39.06</v>
+      </c>
+      <c r="C16" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="22">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="33">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="33">
-        <f>MIBGAS_Spot!E11</f>
+      <c r="B20" s="31">
+        <f>MIBGAS_Spot!E12</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="31">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-07
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -956,10 +956,10 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="13" t="n">
         <v>46302</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="12" t="n">
         <v>75.13</v>
       </c>
       <c r="J12" s="14">
@@ -978,14 +978,11 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E13" s="19">
-        <f>AVERAGE(E6:E12)</f>
-        <v/>
+      <c r="D13" s="16" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>78.27</v>
       </c>
       <c r="J13" s="14">
         <f>A49</f>
@@ -1003,10 +1000,14 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E14" s="19">
+        <f>AVERAGE(E6:E13)</f>
+        <v/>
       </c>
       <c r="J14" s="14">
         <f>A50</f>
@@ -1024,6 +1025,11 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J15" s="14">
         <f>A51</f>
         <v/>
@@ -1078,7 +1084,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E13</f>
+        <f>E14</f>
         <v/>
       </c>
     </row>
@@ -1431,11 +1437,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D15:H15"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1445,7 +1451,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E12">
+  <conditionalFormatting sqref="E6:E13">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1503,7 +1509,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1535,7 +1541,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>76.19</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1553,7 +1559,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>76.7</v>
+        <v>76.37</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1571,7 +1577,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>74.40000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1589,7 +1595,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>73.8</v>
+        <v>76.11</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1607,7 +1613,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>58.95</v>
+        <v>61.25</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1625,7 +1631,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>55.37</v>
+        <v>57.32</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1638,7 +1644,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>54.18</v>
+        <v>56.22</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>57.15</v>
+        <v>57.65</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1664,7 +1670,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>55</v>
+        <v>54.74</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>60.43</v>
+        <v>61.25</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1690,7 +1696,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>39.88</v>
+        <v>40.49</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1729,7 +1735,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E13</f>
+        <f>MIBGAS_Spot!E14</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-08
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -978,10 +978,10 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="13" t="n">
         <v>46303</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="12" t="n">
         <v>78.27</v>
       </c>
       <c r="J13" s="14">
@@ -1000,14 +1000,11 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E14" s="19">
-        <f>AVERAGE(E6:E13)</f>
-        <v/>
+      <c r="D14" s="16" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>78</v>
       </c>
       <c r="J14" s="14">
         <f>A50</f>
@@ -1025,10 +1022,14 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E15" s="19">
+        <f>AVERAGE(E6:E14)</f>
+        <v/>
       </c>
       <c r="J15" s="14">
         <f>A51</f>
@@ -1046,6 +1047,11 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J16" s="14">
         <f>A52</f>
         <v/>
@@ -1084,7 +1090,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E14</f>
+        <f>E15</f>
         <v/>
       </c>
     </row>
@@ -1437,8 +1443,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D15:H15"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D16:H16"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1451,7 +1457,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E13">
+  <conditionalFormatting sqref="E6:E14">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1509,7 +1515,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1541,7 +1547,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>76.29000000000001</v>
+        <v>78.64</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1559,7 +1565,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>76.37</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1577,7 +1583,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>76.5</v>
+        <v>78.18000000000001</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1595,7 +1601,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>76.11</v>
+        <v>77.25</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1613,7 +1619,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>61.25</v>
+        <v>62.06</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1631,7 +1637,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>57.32</v>
+        <v>58.01</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1644,7 +1650,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>56.22</v>
+        <v>56.89</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1657,7 +1663,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>57.65</v>
+        <v>60.25</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1670,7 +1676,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>54.74</v>
+        <v>55.45</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1683,7 +1689,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>61.25</v>
+        <v>63.43</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1696,7 +1702,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>40.49</v>
+        <v>40.82</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1735,7 +1741,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E14</f>
+        <f>MIBGAS_Spot!E15</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-09
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1000,10 +1000,10 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="13" t="n">
         <v>46304</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="12" t="n">
         <v>78</v>
       </c>
       <c r="J14" s="14">
@@ -1022,14 +1022,11 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E15" s="19">
-        <f>AVERAGE(E6:E14)</f>
-        <v/>
+      <c r="D15" s="16" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>80.48999999999999</v>
       </c>
       <c r="J15" s="14">
         <f>A51</f>
@@ -1047,10 +1044,14 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E16" s="19">
+        <f>AVERAGE(E6:E15)</f>
+        <v/>
       </c>
       <c r="J16" s="14">
         <f>A52</f>
@@ -1068,6 +1069,11 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J17" s="14">
         <f>A53</f>
         <v/>
@@ -1090,7 +1096,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E15</f>
+        <f>E16</f>
         <v/>
       </c>
     </row>
@@ -1444,10 +1450,10 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D16:H16"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D17:H17"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1457,7 +1463,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E14">
+  <conditionalFormatting sqref="E6:E15">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1515,7 +1521,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1547,7 +1553,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>78.64</v>
+        <v>77.12</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1565,7 +1571,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>78.09999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1583,7 +1589,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>78.18000000000001</v>
+        <v>76.77</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1601,7 +1607,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>77.25</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1619,7 +1625,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>62.06</v>
+        <v>62.96</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1637,7 +1643,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>58.01</v>
+        <v>58.61</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1650,7 +1656,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>56.89</v>
+        <v>57.02</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1663,7 +1669,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>60.25</v>
+        <v>60.78</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1676,7 +1682,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>55.45</v>
+        <v>55.62</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1689,7 +1695,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>63.43</v>
+        <v>64.48</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1702,7 +1708,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>40.82</v>
+        <v>40.83</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1741,7 +1747,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E15</f>
+        <f>MIBGAS_Spot!E16</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-10
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1022,10 +1022,10 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="13" t="n">
         <v>46305</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="12" t="n">
         <v>80.48999999999999</v>
       </c>
       <c r="J15" s="14">
@@ -1044,14 +1044,11 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E16" s="19">
-        <f>AVERAGE(E6:E15)</f>
-        <v/>
+      <c r="D16" s="16" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>80.90000000000001</v>
       </c>
       <c r="J16" s="14">
         <f>A52</f>
@@ -1069,10 +1066,14 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E17" s="19">
+        <f>AVERAGE(E6:E16)</f>
+        <v/>
       </c>
       <c r="J17" s="14">
         <f>A53</f>
@@ -1090,13 +1091,18 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J18" s="21" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E16</f>
+        <f>E17</f>
         <v/>
       </c>
     </row>
@@ -1453,7 +1459,7 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1463,7 +1469,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E15">
+  <conditionalFormatting sqref="E6:E16">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1747,7 +1753,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E16</f>
+        <f>MIBGAS_Spot!E17</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-11
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -209,13 +209,13 @@
     <xf numFmtId="4" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1044,10 +1044,10 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="16" t="n">
+      <c r="D16" s="13" t="n">
         <v>46306</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="12" t="n">
         <v>80.90000000000001</v>
       </c>
       <c r="J16" s="14">
@@ -1066,14 +1066,11 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E17" s="19">
-        <f>AVERAGE(E6:E16)</f>
-        <v/>
+      <c r="D17" s="16" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>81.18000000000001</v>
       </c>
       <c r="J17" s="14">
         <f>A53</f>
@@ -1091,18 +1088,22 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
-      </c>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E18" s="19">
+        <f>AVERAGE(E6:E17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="K18" s="22">
-        <f>E17</f>
+      <c r="K18" s="21">
+        <f>E18</f>
         <v/>
       </c>
     </row>
@@ -1112,6 +1113,11 @@
       </c>
       <c r="B19" s="12" t="n">
         <v>25.5</v>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1457,9 +1463,9 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D18:H18"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1469,7 +1475,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E16">
+  <conditionalFormatting sqref="E6:E17">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1753,7 +1759,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E17</f>
+        <f>MIBGAS_Spot!E18</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-13
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -199,20 +199,14 @@
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1066,10 +1060,10 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="13" t="n">
         <v>46307</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="12" t="n">
         <v>81.18000000000001</v>
       </c>
       <c r="J17" s="14">
@@ -1088,22 +1082,19 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E18" s="19">
-        <f>AVERAGE(E6:E17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="20" t="inlineStr">
+      <c r="D18" s="13" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>82.89</v>
+      </c>
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="K18" s="21">
-        <f>E18</f>
+      <c r="K18" s="17">
+        <f>E19</f>
         <v/>
       </c>
     </row>
@@ -1114,10 +1105,14 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E19" s="19">
+        <f>AVERAGE(E6:E18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1127,6 +1122,11 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1372,98 +1372,98 @@
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="23" t="n"/>
+      <c r="B51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="23" t="n"/>
+      <c r="B52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="23" t="n"/>
+      <c r="B53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="23" t="n"/>
+      <c r="B56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="23" t="n"/>
+      <c r="B57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="23" t="n"/>
+      <c r="B58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="23" t="n"/>
+      <c r="B59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="23" t="n"/>
+      <c r="B60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="23" t="n"/>
+      <c r="B61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="23" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="23" t="n"/>
+      <c r="B63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="23" t="n"/>
+      <c r="B64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="23" t="n"/>
+      <c r="B65" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D19:H19"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1475,7 +1475,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E17">
+  <conditionalFormatting sqref="E6:E18">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1527,13 +1527,13 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
-        <v>46304</v>
+      <c r="B4" s="23" t="n">
+        <v>46307</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1559,217 +1559,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Mes M+1 (Nov26-Nov26)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
-        <v>77.12</v>
-      </c>
-      <c r="C6" s="28" t="n">
+      <c r="B6" s="25" t="n">
+        <v>82.62</v>
+      </c>
+      <c r="C6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Mes M+2 (Dec26-Dec26)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
-        <v>76.90000000000001</v>
-      </c>
-      <c r="C7" s="28" t="n">
+      <c r="B7" s="25" t="n">
+        <v>83.02</v>
+      </c>
+      <c r="C7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Mes M+3 (Jan27-Jan27)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
-        <v>76.77</v>
-      </c>
-      <c r="C8" s="28" t="n">
+      <c r="B8" s="25" t="n">
+        <v>82.86</v>
+      </c>
+      <c r="C8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
-        <v>75.84999999999999</v>
-      </c>
-      <c r="C9" s="28" t="n">
+      <c r="B9" s="25" t="n">
+        <v>81.76000000000001</v>
+      </c>
+      <c r="C9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
-        <v>62.96</v>
-      </c>
-      <c r="C10" s="28" t="n">
+      <c r="B10" s="25" t="n">
+        <v>63.86</v>
+      </c>
+      <c r="C10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
-        <v>58.61</v>
-      </c>
-      <c r="C11" s="28" t="n">
+      <c r="B11" s="25" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="C11" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Oct27-Dec27)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
-        <v>57.02</v>
-      </c>
-      <c r="C12" s="28" t="n">
+      <c r="B12" s="25" t="n">
+        <v>57.56</v>
+      </c>
+      <c r="C12" s="26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
-        <v>60.78</v>
-      </c>
-      <c r="C13" s="28" t="n">
+      <c r="B13" s="25" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct27-Mar28)</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
-        <v>55.62</v>
-      </c>
-      <c r="C14" s="28" t="n">
+      <c r="B14" s="25" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
-        <v>64.48</v>
-      </c>
-      <c r="C15" s="28" t="n">
+      <c r="B15" s="25" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
-        <v>40.83</v>
-      </c>
-      <c r="C16" s="28" t="n">
+      <c r="B16" s="25" t="n">
+        <v>41.33</v>
+      </c>
+      <c r="C16" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="22">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="33">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="33">
-        <f>MIBGAS_Spot!E18</f>
+      <c r="B20" s="31">
+        <f>MIBGAS_Spot!E19</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="31">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-14
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E20</f>
+        <f>E21</f>
         <v/>
       </c>
     </row>
@@ -1111,10 +1111,10 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="13" t="n">
         <v>46309</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="12" t="n">
         <v>86.3</v>
       </c>
     </row>
@@ -1125,14 +1125,11 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E20" s="21">
-        <f>AVERAGE(E6:E19)</f>
-        <v/>
+      <c r="D20" s="18" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>86.41</v>
       </c>
     </row>
     <row r="21">
@@ -1142,10 +1139,14 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E21" s="21">
+        <f>AVERAGE(E6:E20)</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1155,6 +1156,11 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1472,12 +1478,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D21:H21"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1487,7 +1493,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E19">
+  <conditionalFormatting sqref="E6:E20">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1545,7 +1551,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1577,7 +1583,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>85.20999999999999</v>
+        <v>84.34</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1595,7 +1601,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>86.08</v>
+        <v>84.45999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1613,7 +1619,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>86</v>
+        <v>84.45999999999999</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1631,7 +1637,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>84.84999999999999</v>
+        <v>84.78</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1649,7 +1655,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>65.8</v>
+        <v>66.61</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1667,7 +1673,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>60.94</v>
+        <v>61.87</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1680,7 +1686,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>59.54</v>
+        <v>60.39</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1693,7 +1699,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>63.36</v>
+        <v>64.23</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1706,7 +1712,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>58.15</v>
+        <v>59</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1719,7 +1725,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>67.68000000000001</v>
+        <v>68.33</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1732,7 +1738,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>42.25</v>
+        <v>42.57</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1771,7 +1777,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E20</f>
+        <f>MIBGAS_Spot!E21</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-15
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E21</f>
+        <f>E22</f>
         <v/>
       </c>
     </row>
@@ -1125,10 +1125,10 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="13" t="n">
         <v>46310</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="12" t="n">
         <v>86.41</v>
       </c>
     </row>
@@ -1139,14 +1139,11 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E21" s="21">
-        <f>AVERAGE(E6:E20)</f>
-        <v/>
+      <c r="D21" s="18" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>86.68000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1156,10 +1153,14 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E22" s="21">
+        <f>AVERAGE(E6:E21)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1168,6 +1169,11 @@
       </c>
       <c r="B23" s="12" t="n">
         <v>34.55</v>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1482,8 +1488,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D23:H23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1493,7 +1499,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E20">
+  <conditionalFormatting sqref="E6:E21">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1551,7 +1557,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1583,7 +1589,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>84.34</v>
+        <v>84.88</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1601,7 +1607,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>84.45999999999999</v>
+        <v>85.67</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1619,7 +1625,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>84.45999999999999</v>
+        <v>84.75</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1637,7 +1643,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>84.78</v>
+        <v>83.45</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1655,7 +1661,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>66.61</v>
+        <v>67.59</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1673,7 +1679,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>61.87</v>
+        <v>63.01</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1686,7 +1692,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>60.39</v>
+        <v>61.7</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1699,7 +1705,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>64.23</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1712,7 +1718,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>59</v>
+        <v>60.34</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1725,7 +1731,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>68.33</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1738,7 +1744,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>42.57</v>
+        <v>43.77</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1777,7 +1783,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E21</f>
+        <f>MIBGAS_Spot!E22</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-16
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E22</f>
+        <f>E23</f>
         <v/>
       </c>
     </row>
@@ -1139,10 +1139,10 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="13" t="n">
         <v>46311</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="12" t="n">
         <v>86.68000000000001</v>
       </c>
     </row>
@@ -1153,14 +1153,11 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E22" s="21">
-        <f>AVERAGE(E6:E21)</f>
-        <v/>
+      <c r="D22" s="18" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>86.98999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1170,10 +1167,14 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E23" s="21">
+        <f>AVERAGE(E6:E22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1182,6 +1183,11 @@
       </c>
       <c r="B24" s="12" t="n">
         <v>32.42</v>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1486,9 +1492,9 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D23:H23"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1499,7 +1505,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E21">
+  <conditionalFormatting sqref="E6:E22">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1557,7 +1563,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1589,7 +1595,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>84.88</v>
+        <v>86.72</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1607,7 +1613,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>85.67</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1625,7 +1631,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>84.75</v>
+        <v>86.95</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1643,7 +1649,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>83.45</v>
+        <v>85.92</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1661,7 +1667,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>67.59</v>
+        <v>68.92</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1679,7 +1685,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>63.01</v>
+        <v>64.16</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1692,7 +1698,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>61.7</v>
+        <v>62.35</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1705,7 +1711,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>65.29000000000001</v>
+        <v>66.53</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1718,7 +1724,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>60.34</v>
+        <v>60.97</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1731,7 +1737,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>69.18000000000001</v>
+        <v>69.91</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1744,7 +1750,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>43.77</v>
+        <v>44.31</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1783,7 +1789,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E22</f>
+        <f>MIBGAS_Spot!E23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-17
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E23</f>
+        <f>E24</f>
         <v/>
       </c>
     </row>
@@ -1153,10 +1153,10 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="13" t="n">
         <v>46312</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="12" t="n">
         <v>86.98999999999999</v>
       </c>
     </row>
@@ -1167,14 +1167,11 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E23" s="21">
-        <f>AVERAGE(E6:E22)</f>
-        <v/>
+      <c r="D23" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>88.31999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -1184,10 +1181,14 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E24" s="21">
+        <f>AVERAGE(E6:E23)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1197,6 +1198,11 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1491,8 +1497,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D25:H25"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1505,7 +1511,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E22">
+  <conditionalFormatting sqref="E6:E23">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1789,7 +1795,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E23</f>
+        <f>MIBGAS_Spot!E24</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-18
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E24</f>
+        <f>E25</f>
         <v/>
       </c>
     </row>
@@ -1167,10 +1167,10 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="18" t="n">
+      <c r="D23" s="13" t="n">
         <v>46313</v>
       </c>
-      <c r="E23" s="19" t="n">
+      <c r="E23" s="12" t="n">
         <v>88.31999999999999</v>
       </c>
     </row>
@@ -1181,14 +1181,11 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E24" s="21">
-        <f>AVERAGE(E6:E23)</f>
-        <v/>
+      <c r="D24" s="18" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>89.38</v>
       </c>
     </row>
     <row r="25">
@@ -1198,10 +1195,14 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E25" s="21">
+        <f>AVERAGE(E6:E24)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1211,6 +1212,11 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1497,11 +1503,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D25:H25"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1511,7 +1517,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E23">
+  <conditionalFormatting sqref="E6:E24">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1795,7 +1801,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E24</f>
+        <f>MIBGAS_Spot!E25</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-19
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E25</f>
+        <f>E26</f>
         <v/>
       </c>
     </row>
@@ -1181,10 +1181,10 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="13" t="n">
         <v>46314</v>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E24" s="12" t="n">
         <v>89.38</v>
       </c>
     </row>
@@ -1195,14 +1195,11 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E25" s="21">
-        <f>AVERAGE(E6:E24)</f>
-        <v/>
+      <c r="D25" s="18" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>87.8</v>
       </c>
     </row>
     <row r="26">
@@ -1212,10 +1209,14 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E26" s="21">
+        <f>AVERAGE(E6:E25)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1224,6 +1225,11 @@
       </c>
       <c r="B27" s="12" t="n">
         <v>40.41</v>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1506,8 +1512,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D27:H27"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1517,7 +1523,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E24">
+  <conditionalFormatting sqref="E6:E25">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1575,7 +1581,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1607,7 +1613,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>86.72</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1625,7 +1631,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>87.09999999999999</v>
+        <v>88.08</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1643,7 +1649,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>86.95</v>
+        <v>86.8</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1661,7 +1667,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>85.92</v>
+        <v>86.27</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1679,7 +1685,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>68.92</v>
+        <v>69.61</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1697,7 +1703,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>64.16</v>
+        <v>64.87</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1710,7 +1716,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>62.35</v>
+        <v>62.12</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1723,7 +1729,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>66.53</v>
+        <v>67.23</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1736,7 +1742,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>60.97</v>
+        <v>60.72</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1749,7 +1755,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>69.91</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1762,7 +1768,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>44.31</v>
+        <v>44.1</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1801,7 +1807,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E25</f>
+        <f>MIBGAS_Spot!E26</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-20
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E26</f>
+        <f>E27</f>
         <v/>
       </c>
     </row>
@@ -1195,10 +1195,10 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="13" t="n">
         <v>46315</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="12" t="n">
         <v>87.8</v>
       </c>
     </row>
@@ -1209,14 +1209,11 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E26" s="21">
-        <f>AVERAGE(E6:E25)</f>
-        <v/>
+      <c r="D26" s="18" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>84.84999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -1226,10 +1223,14 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E27" s="21">
+        <f>AVERAGE(E6:E26)</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1238,6 +1239,11 @@
       </c>
       <c r="B28" s="12" t="n">
         <v>44.16</v>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1511,8 +1517,8 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D28:H28"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D27:H27"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1523,7 +1529,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E25">
+  <conditionalFormatting sqref="E6:E26">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1581,7 +1587,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1613,7 +1619,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>87.90000000000001</v>
+        <v>88.09</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1631,7 +1637,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>88.08</v>
+        <v>89.06</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1649,7 +1655,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>86.8</v>
+        <v>88.8</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1667,7 +1673,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>86.27</v>
+        <v>86.79000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1685,7 +1691,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>69.61</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>64.87</v>
+        <v>63.04</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1716,7 +1722,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>62.12</v>
+        <v>61.14</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1729,7 +1735,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>67.23</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1742,7 +1748,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>60.72</v>
+        <v>59.79</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1755,7 +1761,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>71.65000000000001</v>
+        <v>68.33</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1768,7 +1774,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>44.1</v>
+        <v>43.75</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1807,7 +1813,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E26</f>
+        <f>MIBGAS_Spot!E27</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-21
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E27</f>
+        <f>E28</f>
         <v/>
       </c>
     </row>
@@ -1209,10 +1209,10 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="18" t="n">
+      <c r="D26" s="13" t="n">
         <v>46316</v>
       </c>
-      <c r="E26" s="19" t="n">
+      <c r="E26" s="12" t="n">
         <v>84.84999999999999</v>
       </c>
     </row>
@@ -1223,14 +1223,11 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E27" s="21">
-        <f>AVERAGE(E6:E26)</f>
-        <v/>
+      <c r="D27" s="18" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>86.73</v>
       </c>
     </row>
     <row r="28">
@@ -1240,10 +1237,14 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E28" s="21">
+        <f>AVERAGE(E6:E27)</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1252,6 +1253,11 @@
       </c>
       <c r="B29" s="12" t="n">
         <v>46.23</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1517,8 +1523,8 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D28:H28"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1529,7 +1535,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E26">
+  <conditionalFormatting sqref="E6:E27">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1587,7 +1593,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1619,7 +1625,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>88.09</v>
+        <v>86.83</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1637,7 +1643,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>89.06</v>
+        <v>86.43000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1655,7 +1661,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>88.8</v>
+        <v>87.13</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1673,7 +1679,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>86.79000000000001</v>
+        <v>85.01000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1691,7 +1697,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>67.29000000000001</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1709,7 +1715,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>63.04</v>
+        <v>66.06</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1722,7 +1728,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>61.14</v>
+        <v>63.94</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1735,7 +1741,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>65.15000000000001</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1748,7 +1754,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>59.79</v>
+        <v>62.47</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1761,7 +1767,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>68.33</v>
+        <v>71.23</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1774,7 +1780,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>43.75</v>
+        <v>45.4</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1813,7 +1819,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E27</f>
+        <f>MIBGAS_Spot!E28</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-22
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E28</f>
+        <f>E29</f>
         <v/>
       </c>
     </row>
@@ -1223,10 +1223,10 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="13" t="n">
         <v>46317</v>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E27" s="12" t="n">
         <v>86.73</v>
       </c>
     </row>
@@ -1237,14 +1237,11 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E28" s="21">
-        <f>AVERAGE(E6:E27)</f>
-        <v/>
+      <c r="D28" s="18" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>89.18000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1254,10 +1251,14 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E29" s="21">
+        <f>AVERAGE(E6:E28)</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1267,6 +1268,11 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -1520,11 +1526,11 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D30:H30"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1535,7 +1541,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E27">
+  <conditionalFormatting sqref="E6:E28">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1593,7 +1599,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1625,7 +1631,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>86.83</v>
+        <v>88.95999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1643,7 +1649,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>86.43000000000001</v>
+        <v>89.19</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1661,7 +1667,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>87.13</v>
+        <v>89.11</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1679,7 +1685,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>85.01000000000001</v>
+        <v>87.84999999999999</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1697,7 +1703,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>70.31999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1715,7 +1721,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>66.06</v>
+        <v>67.28</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1728,7 +1734,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>63.94</v>
+        <v>65.11</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1741,7 +1747,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>68.18000000000001</v>
+        <v>69.48</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1754,7 +1760,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>62.47</v>
+        <v>63.66</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1767,7 +1773,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>71.23</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1780,7 +1786,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>45.4</v>
+        <v>46.35</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1819,7 +1825,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E28</f>
+        <f>MIBGAS_Spot!E29</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-23
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E29</f>
+        <f>E30</f>
         <v/>
       </c>
     </row>
@@ -1237,10 +1237,10 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="18" t="n">
+      <c r="D28" s="13" t="n">
         <v>46318</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="12" t="n">
         <v>89.18000000000001</v>
       </c>
     </row>
@@ -1251,14 +1251,11 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E29" s="21">
-        <f>AVERAGE(E6:E28)</f>
-        <v/>
+      <c r="D29" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E29" s="19" t="n">
+        <v>92.53</v>
       </c>
     </row>
     <row r="30">
@@ -1268,10 +1265,14 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E30" s="21">
+        <f>AVERAGE(E6:E29)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1281,6 +1282,11 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1526,12 +1532,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D30:H30"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1541,7 +1547,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E28">
+  <conditionalFormatting sqref="E6:E29">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1599,7 +1605,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1631,7 +1637,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>88.95999999999999</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1649,7 +1655,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>89.19</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1667,7 +1673,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>89.11</v>
+        <v>92.8</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1685,7 +1691,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>87.84999999999999</v>
+        <v>91.59</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>71.7</v>
+        <v>73.45</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1721,7 +1727,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>67.28</v>
+        <v>68.63</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1734,7 +1740,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>65.11</v>
+        <v>66.63</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1747,7 +1753,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>69.48</v>
+        <v>71.5</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1760,7 +1766,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>63.66</v>
+        <v>65.11</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1773,7 +1779,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>72.93000000000001</v>
+        <v>76</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1786,7 +1792,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>46.35</v>
+        <v>48.45</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1825,7 +1831,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E29</f>
+        <f>MIBGAS_Spot!E30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-24
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E30</f>
+        <f>E31</f>
         <v/>
       </c>
     </row>
@@ -1251,10 +1251,10 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="18" t="n">
+      <c r="D29" s="13" t="n">
         <v>46319</v>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E29" s="12" t="n">
         <v>92.53</v>
       </c>
     </row>
@@ -1265,14 +1265,11 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E30" s="21">
-        <f>AVERAGE(E6:E29)</f>
-        <v/>
+      <c r="D30" s="18" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E30" s="19" t="n">
+        <v>99.38</v>
       </c>
     </row>
     <row r="31">
@@ -1282,10 +1279,14 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E31" s="21">
+        <f>AVERAGE(E6:E30)</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1294,6 +1295,11 @@
       </c>
       <c r="B32" s="12" t="n">
         <v>41.41</v>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1537,7 +1543,7 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1547,7 +1553,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E29">
+  <conditionalFormatting sqref="E6:E30">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1831,7 +1837,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E30</f>
+        <f>MIBGAS_Spot!E31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-25
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E31</f>
+        <f>E32</f>
         <v/>
       </c>
     </row>
@@ -1265,10 +1265,10 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="13" t="n">
         <v>46320</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="12" t="n">
         <v>99.38</v>
       </c>
     </row>
@@ -1279,14 +1279,11 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E31" s="21">
-        <f>AVERAGE(E6:E30)</f>
-        <v/>
+      <c r="D31" s="18" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>97.08</v>
       </c>
     </row>
     <row r="32">
@@ -1296,10 +1293,14 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E32" s="21">
+        <f>AVERAGE(E6:E31)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1308,6 +1309,11 @@
       </c>
       <c r="B33" s="12" t="n">
         <v>33.76</v>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1541,9 +1547,9 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D33:H33"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D32:H32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1553,7 +1559,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E30">
+  <conditionalFormatting sqref="E6:E31">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1837,7 +1843,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E31</f>
+        <f>MIBGAS_Spot!E32</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-26
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E32</f>
+        <f>E33</f>
         <v/>
       </c>
     </row>
@@ -1279,10 +1279,10 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="13" t="n">
         <v>46321</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="12" t="n">
         <v>97.08</v>
       </c>
     </row>
@@ -1293,14 +1293,11 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E32" s="21">
-        <f>AVERAGE(E6:E31)</f>
-        <v/>
+      <c r="D32" s="18" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>95.93000000000001</v>
       </c>
     </row>
     <row r="33">
@@ -1310,10 +1307,14 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E33" s="21">
+        <f>AVERAGE(E6:E32)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1322,6 +1323,11 @@
       </c>
       <c r="B34" s="12" t="n">
         <v>34.02</v>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1546,8 +1552,8 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D34:H34"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D33:H33"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1559,7 +1565,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E31">
+  <conditionalFormatting sqref="E6:E32">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1617,7 +1623,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1649,7 +1655,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>92.59999999999999</v>
+        <v>95.19</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1667,7 +1673,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>92.65000000000001</v>
+        <v>95.28</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1685,7 +1691,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>92.8</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>91.59</v>
+        <v>93.83</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1721,7 +1727,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>73.45</v>
+        <v>75.75</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1739,7 +1745,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>68.63</v>
+        <v>70.73</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1752,7 +1758,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>66.63</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1765,7 +1771,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>71.5</v>
+        <v>73.23</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1778,7 +1784,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>65.11</v>
+        <v>67.41</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1791,7 +1797,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>76</v>
+        <v>77.33</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1804,7 +1810,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>48.45</v>
+        <v>48.7</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1843,7 +1849,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E32</f>
+        <f>MIBGAS_Spot!E33</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-27
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E33</f>
+        <f>E34</f>
         <v/>
       </c>
     </row>
@@ -1293,10 +1293,10 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="18" t="n">
+      <c r="D32" s="13" t="n">
         <v>46322</v>
       </c>
-      <c r="E32" s="19" t="n">
+      <c r="E32" s="12" t="n">
         <v>95.93000000000001</v>
       </c>
     </row>
@@ -1307,14 +1307,11 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E33" s="21">
-        <f>AVERAGE(E6:E32)</f>
-        <v/>
+      <c r="D33" s="18" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E33" s="19" t="n">
+        <v>95.5</v>
       </c>
     </row>
     <row r="34">
@@ -1324,10 +1321,14 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D34" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E34" s="21">
+        <f>AVERAGE(E6:E33)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -1337,6 +1338,11 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1550,9 +1556,9 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D35:H35"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D34:H34"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1565,7 +1571,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E32">
+  <conditionalFormatting sqref="E6:E33">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1623,7 +1629,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1655,7 +1661,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>95.19</v>
+        <v>93.81999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1673,7 +1679,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>95.28</v>
+        <v>95.03</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1691,7 +1697,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>95.54000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1709,7 +1715,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>93.83</v>
+        <v>91.63</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1727,7 +1733,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>75.75</v>
+        <v>74.09</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1745,7 +1751,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>70.73</v>
+        <v>69.19</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1758,7 +1764,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>68.90000000000001</v>
+        <v>67.67</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1771,7 +1777,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>73.23</v>
+        <v>71.63</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1784,7 +1790,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>67.41</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1797,7 +1803,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>77.33</v>
+        <v>75.68000000000001</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1810,7 +1816,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>48.7</v>
+        <v>48.28</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1849,7 +1855,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E33</f>
+        <f>MIBGAS_Spot!E34</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-28
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E34</f>
+        <f>E35</f>
         <v/>
       </c>
     </row>
@@ -1307,10 +1307,10 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="18" t="n">
+      <c r="D33" s="13" t="n">
         <v>46323</v>
       </c>
-      <c r="E33" s="19" t="n">
+      <c r="E33" s="12" t="n">
         <v>95.5</v>
       </c>
     </row>
@@ -1321,14 +1321,11 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E34" s="21">
-        <f>AVERAGE(E6:E33)</f>
-        <v/>
+      <c r="D34" s="18" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <v>99.92</v>
       </c>
     </row>
     <row r="35">
@@ -1338,10 +1335,14 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D35" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E35" s="21">
+        <f>AVERAGE(E6:E34)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -1351,6 +1352,11 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1556,12 +1562,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D35:H35"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D36:H36"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1571,7 +1577,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E33">
+  <conditionalFormatting sqref="E6:E34">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1629,7 +1635,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1661,7 +1667,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>93.81999999999999</v>
+        <v>98.06</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1679,7 +1685,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>95.03</v>
+        <v>96.7</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1697,7 +1703,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>93.7</v>
+        <v>98.77</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1715,7 +1721,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>91.63</v>
+        <v>96.94</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1733,7 +1739,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>74.09</v>
+        <v>77</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1751,7 +1757,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>69.19</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1764,7 +1770,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>67.67</v>
+        <v>70</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1777,7 +1783,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>71.63</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1790,7 +1796,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>66.20999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1803,7 +1809,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>75.68000000000001</v>
+        <v>78.38</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1816,7 +1822,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>48.28</v>
+        <v>49.37</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1855,7 +1861,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E34</f>
+        <f>MIBGAS_Spot!E35</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-29
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E35</f>
+        <f>E36</f>
         <v/>
       </c>
     </row>
@@ -1321,10 +1321,10 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="18" t="n">
+      <c r="D34" s="13" t="n">
         <v>46324</v>
       </c>
-      <c r="E34" s="19" t="n">
+      <c r="E34" s="12" t="n">
         <v>99.92</v>
       </c>
     </row>
@@ -1335,14 +1335,11 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E35" s="21">
-        <f>AVERAGE(E6:E34)</f>
-        <v/>
+      <c r="D35" s="18" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E35" s="19" t="n">
+        <v>97.84999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -1352,10 +1349,14 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D36" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E36" s="21">
+        <f>AVERAGE(E6:E35)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1364,6 +1365,11 @@
       </c>
       <c r="B37" s="12" t="n">
         <v>32.58</v>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1566,8 +1572,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D37:H37"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D36:H36"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1577,7 +1583,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E34">
+  <conditionalFormatting sqref="E6:E35">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1635,7 +1641,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1667,7 +1673,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>98.06</v>
+        <v>96.13</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1685,7 +1691,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>96.7</v>
+        <v>96.45</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>98.77</v>
+        <v>96.84999999999999</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1721,7 +1727,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>96.94</v>
+        <v>94.15000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1739,7 +1745,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>77</v>
+        <v>74.38</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1757,7 +1763,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>71.01000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1770,7 +1776,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>70</v>
+        <v>66.5</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1783,7 +1789,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>73.68000000000001</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1796,7 +1802,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>67.7</v>
+        <v>65.02</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1809,7 +1815,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>78.38</v>
+        <v>76.33</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1822,7 +1828,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>49.37</v>
+        <v>47.45</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1861,7 +1867,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E35</f>
+        <f>MIBGAS_Spot!E36</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-10-30
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E36</f>
+        <f>E37</f>
         <v/>
       </c>
     </row>
@@ -1335,10 +1335,10 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="18" t="n">
+      <c r="D35" s="13" t="n">
         <v>46325</v>
       </c>
-      <c r="E35" s="19" t="n">
+      <c r="E35" s="12" t="n">
         <v>97.84999999999999</v>
       </c>
     </row>
@@ -1349,14 +1349,11 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E36" s="21">
-        <f>AVERAGE(E6:E35)</f>
-        <v/>
+      <c r="D36" s="18" t="n">
+        <v>46326</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>103.49</v>
       </c>
     </row>
     <row r="37">
@@ -1366,10 +1363,14 @@
       <c r="B37" s="12" t="n">
         <v>32.58</v>
       </c>
-      <c r="D37" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E37" s="21">
+        <f>AVERAGE(E6:E36)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1378,6 +1379,11 @@
       </c>
       <c r="B38" s="12" t="n">
         <v>31.84</v>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1572,7 +1578,7 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1583,7 +1589,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E35">
+  <conditionalFormatting sqref="E6:E36">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1641,7 +1647,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1673,7 +1679,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>96.13</v>
+        <v>102.66</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1691,7 +1697,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>96.45</v>
+        <v>101.6</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>1</v>
@@ -1709,7 +1715,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>96.84999999999999</v>
+        <v>101.69</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1727,7 +1733,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>94.15000000000001</v>
+        <v>100.08</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1745,7 +1751,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>74.38</v>
+        <v>77.94</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1763,7 +1769,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>69.5</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1776,7 +1782,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>66.5</v>
+        <v>70.2</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>1</v>
@@ -1789,7 +1795,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>71.93000000000001</v>
+        <v>75.16</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1802,7 +1808,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>65.02</v>
+        <v>68.5</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1815,7 +1821,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>76.33</v>
+        <v>80.5</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1828,7 +1834,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>47.45</v>
+        <v>49.4</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1867,7 +1873,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E36</f>
+        <f>MIBGAS_Spot!E37</f>
         <v/>
       </c>
     </row>

</xml_diff>